<commit_message>
chore(data): sync FEB data 2026-04-27 13:27
</commit_message>
<xml_diff>
--- a/data/1FEB_25_26/players_25_26_1FEB_games.xlsx
+++ b/data/1FEB_25_26/players_25_26_1FEB_games.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI481"/>
+  <dimension ref="A1:AI513"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57723,6 +57723,3814 @@
       </c>
       <c r="AI481" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B482" t="n">
+        <v>31</v>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>200</v>
+      </c>
+      <c r="F482" t="n">
+        <v>89</v>
+      </c>
+      <c r="G482" t="n">
+        <v>20</v>
+      </c>
+      <c r="H482" t="n">
+        <v>34</v>
+      </c>
+      <c r="I482" t="n">
+        <v>14</v>
+      </c>
+      <c r="J482" t="n">
+        <v>36</v>
+      </c>
+      <c r="K482" t="n">
+        <v>7</v>
+      </c>
+      <c r="L482" t="n">
+        <v>14</v>
+      </c>
+      <c r="M482" t="n">
+        <v>15</v>
+      </c>
+      <c r="N482" t="n">
+        <v>24</v>
+      </c>
+      <c r="O482" t="n">
+        <v>23</v>
+      </c>
+      <c r="P482" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q482" t="n">
+        <v>9</v>
+      </c>
+      <c r="R482" t="n">
+        <v>18</v>
+      </c>
+      <c r="S482" t="n">
+        <v>19</v>
+      </c>
+      <c r="T482" t="n">
+        <v>0</v>
+      </c>
+      <c r="U482" t="inlineStr">
+        <is>
+          <t>2486535</t>
+        </is>
+      </c>
+      <c r="V482" t="n">
+        <v>74</v>
+      </c>
+      <c r="W482" t="n">
+        <v>85.16</v>
+      </c>
+      <c r="X482" t="n">
+        <v>1.045091592296853</v>
+      </c>
+      <c r="Y482" t="n">
+        <v>70.16</v>
+      </c>
+      <c r="Z482" t="n">
+        <v>126.8529076396807</v>
+      </c>
+      <c r="AA482" t="n">
+        <v>0.9245377311344328</v>
+      </c>
+      <c r="AB482" t="n">
+        <v>99.94597514856835</v>
+      </c>
+      <c r="AC482" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="AD482" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AE482" t="n">
+        <v>0.5909090909090909</v>
+      </c>
+      <c r="AF482" t="n">
+        <v>26.90693249111239</v>
+      </c>
+      <c r="AG482" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="AH482" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="AI482" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B483" t="n">
+        <v>31</v>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>200</v>
+      </c>
+      <c r="F483" t="n">
+        <v>78</v>
+      </c>
+      <c r="G483" t="n">
+        <v>19</v>
+      </c>
+      <c r="H483" t="n">
+        <v>45</v>
+      </c>
+      <c r="I483" t="n">
+        <v>8</v>
+      </c>
+      <c r="J483" t="n">
+        <v>22</v>
+      </c>
+      <c r="K483" t="n">
+        <v>16</v>
+      </c>
+      <c r="L483" t="n">
+        <v>19</v>
+      </c>
+      <c r="M483" t="n">
+        <v>12</v>
+      </c>
+      <c r="N483" t="n">
+        <v>29</v>
+      </c>
+      <c r="O483" t="n">
+        <v>15</v>
+      </c>
+      <c r="P483" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q483" t="n">
+        <v>16</v>
+      </c>
+      <c r="R483" t="n">
+        <v>21</v>
+      </c>
+      <c r="S483" t="n">
+        <v>20</v>
+      </c>
+      <c r="T483" t="n">
+        <v>2</v>
+      </c>
+      <c r="U483" t="inlineStr">
+        <is>
+          <t>2486533</t>
+        </is>
+      </c>
+      <c r="V483" t="n">
+        <v>64</v>
+      </c>
+      <c r="W483" t="n">
+        <v>91.36</v>
+      </c>
+      <c r="X483" t="n">
+        <v>0.8537653239929948</v>
+      </c>
+      <c r="Y483" t="n">
+        <v>79.36</v>
+      </c>
+      <c r="Z483" t="n">
+        <v>98.28629032258064</v>
+      </c>
+      <c r="AA483" t="n">
+        <v>0.7191011235955056</v>
+      </c>
+      <c r="AB483" t="n">
+        <v>81.01265822784811</v>
+      </c>
+      <c r="AC483" t="n">
+        <v>0.3157894736842105</v>
+      </c>
+      <c r="AD483" t="n">
+        <v>0.7435897435897436</v>
+      </c>
+      <c r="AE483" t="n">
+        <v>0.5324675324675324</v>
+      </c>
+      <c r="AF483" t="n">
+        <v>17.27363209473253</v>
+      </c>
+      <c r="AG483" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="AH483" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="AI483" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B484" t="n">
+        <v>31</v>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>200</v>
+      </c>
+      <c r="F484" t="n">
+        <v>90</v>
+      </c>
+      <c r="G484" t="n">
+        <v>22</v>
+      </c>
+      <c r="H484" t="n">
+        <v>36</v>
+      </c>
+      <c r="I484" t="n">
+        <v>10</v>
+      </c>
+      <c r="J484" t="n">
+        <v>25</v>
+      </c>
+      <c r="K484" t="n">
+        <v>16</v>
+      </c>
+      <c r="L484" t="n">
+        <v>26</v>
+      </c>
+      <c r="M484" t="n">
+        <v>13</v>
+      </c>
+      <c r="N484" t="n">
+        <v>24</v>
+      </c>
+      <c r="O484" t="n">
+        <v>20</v>
+      </c>
+      <c r="P484" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q484" t="n">
+        <v>14</v>
+      </c>
+      <c r="R484" t="n">
+        <v>24</v>
+      </c>
+      <c r="S484" t="n">
+        <v>25</v>
+      </c>
+      <c r="T484" t="n">
+        <v>2</v>
+      </c>
+      <c r="U484" t="inlineStr">
+        <is>
+          <t>2486534</t>
+        </is>
+      </c>
+      <c r="V484" t="n">
+        <v>93</v>
+      </c>
+      <c r="W484" t="n">
+        <v>86.44</v>
+      </c>
+      <c r="X484" t="n">
+        <v>1.041184636742249</v>
+      </c>
+      <c r="Y484" t="n">
+        <v>73.44</v>
+      </c>
+      <c r="Z484" t="n">
+        <v>122.5490196078431</v>
+      </c>
+      <c r="AA484" t="n">
+        <v>1.085941148995796</v>
+      </c>
+      <c r="AB484" t="n">
+        <v>118.2604272634791</v>
+      </c>
+      <c r="AC484" t="n">
+        <v>0.4193548387096774</v>
+      </c>
+      <c r="AD484" t="n">
+        <v>0.7741935483870968</v>
+      </c>
+      <c r="AE484" t="n">
+        <v>0.5967741935483871</v>
+      </c>
+      <c r="AF484" t="n">
+        <v>4.288592344363991</v>
+      </c>
+      <c r="AG484" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="AH484" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="AI484" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B485" t="n">
+        <v>31</v>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>200</v>
+      </c>
+      <c r="F485" t="n">
+        <v>63</v>
+      </c>
+      <c r="G485" t="n">
+        <v>15</v>
+      </c>
+      <c r="H485" t="n">
+        <v>42</v>
+      </c>
+      <c r="I485" t="n">
+        <v>8</v>
+      </c>
+      <c r="J485" t="n">
+        <v>23</v>
+      </c>
+      <c r="K485" t="n">
+        <v>9</v>
+      </c>
+      <c r="L485" t="n">
+        <v>14</v>
+      </c>
+      <c r="M485" t="n">
+        <v>10</v>
+      </c>
+      <c r="N485" t="n">
+        <v>19</v>
+      </c>
+      <c r="O485" t="n">
+        <v>15</v>
+      </c>
+      <c r="P485" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q485" t="n">
+        <v>9</v>
+      </c>
+      <c r="R485" t="n">
+        <v>18</v>
+      </c>
+      <c r="S485" t="n">
+        <v>17</v>
+      </c>
+      <c r="T485" t="n">
+        <v>1</v>
+      </c>
+      <c r="U485" t="inlineStr">
+        <is>
+          <t>2486529</t>
+        </is>
+      </c>
+      <c r="V485" t="n">
+        <v>73</v>
+      </c>
+      <c r="W485" t="n">
+        <v>80.16</v>
+      </c>
+      <c r="X485" t="n">
+        <v>0.7859281437125749</v>
+      </c>
+      <c r="Y485" t="n">
+        <v>70.16</v>
+      </c>
+      <c r="Z485" t="n">
+        <v>89.79475484606614</v>
+      </c>
+      <c r="AA485" t="n">
+        <v>0.9843581445523194</v>
+      </c>
+      <c r="AB485" t="n">
+        <v>110.3385731559855</v>
+      </c>
+      <c r="AC485" t="n">
+        <v>0.2702702702702703</v>
+      </c>
+      <c r="AD485" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="AE485" t="n">
+        <v>0.453125</v>
+      </c>
+      <c r="AF485" t="n">
+        <v>-20.54381830991936</v>
+      </c>
+      <c r="AG485" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="AH485" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="AI485" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B486" t="n">
+        <v>31</v>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>200</v>
+      </c>
+      <c r="F486" t="n">
+        <v>89</v>
+      </c>
+      <c r="G486" t="n">
+        <v>24</v>
+      </c>
+      <c r="H486" t="n">
+        <v>44</v>
+      </c>
+      <c r="I486" t="n">
+        <v>7</v>
+      </c>
+      <c r="J486" t="n">
+        <v>20</v>
+      </c>
+      <c r="K486" t="n">
+        <v>20</v>
+      </c>
+      <c r="L486" t="n">
+        <v>21</v>
+      </c>
+      <c r="M486" t="n">
+        <v>4</v>
+      </c>
+      <c r="N486" t="n">
+        <v>26</v>
+      </c>
+      <c r="O486" t="n">
+        <v>20</v>
+      </c>
+      <c r="P486" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q486" t="n">
+        <v>9</v>
+      </c>
+      <c r="R486" t="n">
+        <v>18</v>
+      </c>
+      <c r="S486" t="n">
+        <v>21</v>
+      </c>
+      <c r="T486" t="n">
+        <v>1</v>
+      </c>
+      <c r="U486" t="inlineStr">
+        <is>
+          <t>2486536</t>
+        </is>
+      </c>
+      <c r="V486" t="n">
+        <v>80</v>
+      </c>
+      <c r="W486" t="n">
+        <v>82.24000000000001</v>
+      </c>
+      <c r="X486" t="n">
+        <v>1.082198443579766</v>
+      </c>
+      <c r="Y486" t="n">
+        <v>78.24000000000001</v>
+      </c>
+      <c r="Z486" t="n">
+        <v>113.7525562372188</v>
+      </c>
+      <c r="AA486" t="n">
+        <v>0.9737098344693281</v>
+      </c>
+      <c r="AB486" t="n">
+        <v>103.6806635562468</v>
+      </c>
+      <c r="AC486" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="AD486" t="n">
+        <v>0.8387096774193549</v>
+      </c>
+      <c r="AE486" t="n">
+        <v>0.4918032786885246</v>
+      </c>
+      <c r="AF486" t="n">
+        <v>10.07189268097203</v>
+      </c>
+      <c r="AG486" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="AH486" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="AI486" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B487" t="n">
+        <v>31</v>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>200</v>
+      </c>
+      <c r="F487" t="n">
+        <v>80</v>
+      </c>
+      <c r="G487" t="n">
+        <v>16</v>
+      </c>
+      <c r="H487" t="n">
+        <v>30</v>
+      </c>
+      <c r="I487" t="n">
+        <v>13</v>
+      </c>
+      <c r="J487" t="n">
+        <v>32</v>
+      </c>
+      <c r="K487" t="n">
+        <v>9</v>
+      </c>
+      <c r="L487" t="n">
+        <v>14</v>
+      </c>
+      <c r="M487" t="n">
+        <v>5</v>
+      </c>
+      <c r="N487" t="n">
+        <v>26</v>
+      </c>
+      <c r="O487" t="n">
+        <v>20</v>
+      </c>
+      <c r="P487" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q487" t="n">
+        <v>14</v>
+      </c>
+      <c r="R487" t="n">
+        <v>21</v>
+      </c>
+      <c r="S487" t="n">
+        <v>16</v>
+      </c>
+      <c r="T487" t="n">
+        <v>2</v>
+      </c>
+      <c r="U487" t="inlineStr">
+        <is>
+          <t>2486536</t>
+        </is>
+      </c>
+      <c r="V487" t="n">
+        <v>89</v>
+      </c>
+      <c r="W487" t="n">
+        <v>82.16</v>
+      </c>
+      <c r="X487" t="n">
+        <v>0.9737098344693281</v>
+      </c>
+      <c r="Y487" t="n">
+        <v>77.16</v>
+      </c>
+      <c r="Z487" t="n">
+        <v>103.6806635562468</v>
+      </c>
+      <c r="AA487" t="n">
+        <v>1.082198443579766</v>
+      </c>
+      <c r="AB487" t="n">
+        <v>113.7525562372188</v>
+      </c>
+      <c r="AC487" t="n">
+        <v>0.1612903225806452</v>
+      </c>
+      <c r="AD487" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="AE487" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="AF487" t="n">
+        <v>-10.07189268097203</v>
+      </c>
+      <c r="AG487" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="AH487" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="AI487" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B488" t="n">
+        <v>31</v>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>200</v>
+      </c>
+      <c r="F488" t="n">
+        <v>64</v>
+      </c>
+      <c r="G488" t="n">
+        <v>14</v>
+      </c>
+      <c r="H488" t="n">
+        <v>26</v>
+      </c>
+      <c r="I488" t="n">
+        <v>7</v>
+      </c>
+      <c r="J488" t="n">
+        <v>35</v>
+      </c>
+      <c r="K488" t="n">
+        <v>15</v>
+      </c>
+      <c r="L488" t="n">
+        <v>25</v>
+      </c>
+      <c r="M488" t="n">
+        <v>10</v>
+      </c>
+      <c r="N488" t="n">
+        <v>26</v>
+      </c>
+      <c r="O488" t="n">
+        <v>17</v>
+      </c>
+      <c r="P488" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q488" t="n">
+        <v>17</v>
+      </c>
+      <c r="R488" t="n">
+        <v>20</v>
+      </c>
+      <c r="S488" t="n">
+        <v>21</v>
+      </c>
+      <c r="T488" t="n">
+        <v>4</v>
+      </c>
+      <c r="U488" t="inlineStr">
+        <is>
+          <t>2486533</t>
+        </is>
+      </c>
+      <c r="V488" t="n">
+        <v>78</v>
+      </c>
+      <c r="W488" t="n">
+        <v>89</v>
+      </c>
+      <c r="X488" t="n">
+        <v>0.7191011235955056</v>
+      </c>
+      <c r="Y488" t="n">
+        <v>79</v>
+      </c>
+      <c r="Z488" t="n">
+        <v>81.01265822784811</v>
+      </c>
+      <c r="AA488" t="n">
+        <v>0.8537653239929948</v>
+      </c>
+      <c r="AB488" t="n">
+        <v>98.28629032258064</v>
+      </c>
+      <c r="AC488" t="n">
+        <v>0.2564102564102564</v>
+      </c>
+      <c r="AD488" t="n">
+        <v>0.6842105263157895</v>
+      </c>
+      <c r="AE488" t="n">
+        <v>0.4675324675324675</v>
+      </c>
+      <c r="AF488" t="n">
+        <v>-17.27363209473253</v>
+      </c>
+      <c r="AG488" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="AH488" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="AI488" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B489" t="n">
+        <v>31</v>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>225</v>
+      </c>
+      <c r="F489" t="n">
+        <v>99</v>
+      </c>
+      <c r="G489" t="n">
+        <v>18</v>
+      </c>
+      <c r="H489" t="n">
+        <v>36</v>
+      </c>
+      <c r="I489" t="n">
+        <v>16</v>
+      </c>
+      <c r="J489" t="n">
+        <v>35</v>
+      </c>
+      <c r="K489" t="n">
+        <v>15</v>
+      </c>
+      <c r="L489" t="n">
+        <v>20</v>
+      </c>
+      <c r="M489" t="n">
+        <v>3</v>
+      </c>
+      <c r="N489" t="n">
+        <v>24</v>
+      </c>
+      <c r="O489" t="n">
+        <v>15</v>
+      </c>
+      <c r="P489" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q489" t="n">
+        <v>12</v>
+      </c>
+      <c r="R489" t="n">
+        <v>21</v>
+      </c>
+      <c r="S489" t="n">
+        <v>19</v>
+      </c>
+      <c r="T489" t="n">
+        <v>1</v>
+      </c>
+      <c r="U489" t="inlineStr">
+        <is>
+          <t>2486530</t>
+        </is>
+      </c>
+      <c r="V489" t="n">
+        <v>96</v>
+      </c>
+      <c r="W489" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="X489" t="n">
+        <v>1.07843137254902</v>
+      </c>
+      <c r="Y489" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="Z489" t="n">
+        <v>111.4864864864865</v>
+      </c>
+      <c r="AA489" t="n">
+        <v>0.9696969696969697</v>
+      </c>
+      <c r="AB489" t="n">
+        <v>109.0909090909091</v>
+      </c>
+      <c r="AC489" t="n">
+        <v>0.09375</v>
+      </c>
+      <c r="AD489" t="n">
+        <v>0.6857142857142857</v>
+      </c>
+      <c r="AE489" t="n">
+        <v>0.4029850746268657</v>
+      </c>
+      <c r="AF489" t="n">
+        <v>2.395577395577391</v>
+      </c>
+      <c r="AG489" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="AH489" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="AI489" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B490" t="n">
+        <v>31</v>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>200</v>
+      </c>
+      <c r="F490" t="n">
+        <v>72</v>
+      </c>
+      <c r="G490" t="n">
+        <v>15</v>
+      </c>
+      <c r="H490" t="n">
+        <v>35</v>
+      </c>
+      <c r="I490" t="n">
+        <v>10</v>
+      </c>
+      <c r="J490" t="n">
+        <v>27</v>
+      </c>
+      <c r="K490" t="n">
+        <v>12</v>
+      </c>
+      <c r="L490" t="n">
+        <v>17</v>
+      </c>
+      <c r="M490" t="n">
+        <v>8</v>
+      </c>
+      <c r="N490" t="n">
+        <v>20</v>
+      </c>
+      <c r="O490" t="n">
+        <v>13</v>
+      </c>
+      <c r="P490" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q490" t="n">
+        <v>9</v>
+      </c>
+      <c r="R490" t="n">
+        <v>27</v>
+      </c>
+      <c r="S490" t="n">
+        <v>22</v>
+      </c>
+      <c r="T490" t="n">
+        <v>2</v>
+      </c>
+      <c r="U490" t="inlineStr">
+        <is>
+          <t>2486531</t>
+        </is>
+      </c>
+      <c r="V490" t="n">
+        <v>81</v>
+      </c>
+      <c r="W490" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="X490" t="n">
+        <v>0.9174311926605504</v>
+      </c>
+      <c r="Y490" t="n">
+        <v>70.48</v>
+      </c>
+      <c r="Z490" t="n">
+        <v>102.1566401816118</v>
+      </c>
+      <c r="AA490" t="n">
+        <v>0.9839650145772596</v>
+      </c>
+      <c r="AB490" t="n">
+        <v>113.5726303982053</v>
+      </c>
+      <c r="AC490" t="n">
+        <v>0.2352941176470588</v>
+      </c>
+      <c r="AD490" t="n">
+        <v>0.6451612903225806</v>
+      </c>
+      <c r="AE490" t="n">
+        <v>0.4307692307692308</v>
+      </c>
+      <c r="AF490" t="n">
+        <v>-11.41599021659347</v>
+      </c>
+      <c r="AG490" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="AH490" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="AI490" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B491" t="n">
+        <v>31</v>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>200</v>
+      </c>
+      <c r="F491" t="n">
+        <v>73</v>
+      </c>
+      <c r="G491" t="n">
+        <v>26</v>
+      </c>
+      <c r="H491" t="n">
+        <v>42</v>
+      </c>
+      <c r="I491" t="n">
+        <v>4</v>
+      </c>
+      <c r="J491" t="n">
+        <v>18</v>
+      </c>
+      <c r="K491" t="n">
+        <v>9</v>
+      </c>
+      <c r="L491" t="n">
+        <v>14</v>
+      </c>
+      <c r="M491" t="n">
+        <v>8</v>
+      </c>
+      <c r="N491" t="n">
+        <v>27</v>
+      </c>
+      <c r="O491" t="n">
+        <v>23</v>
+      </c>
+      <c r="P491" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q491" t="n">
+        <v>8</v>
+      </c>
+      <c r="R491" t="n">
+        <v>18</v>
+      </c>
+      <c r="S491" t="n">
+        <v>18</v>
+      </c>
+      <c r="T491" t="n">
+        <v>6</v>
+      </c>
+      <c r="U491" t="inlineStr">
+        <is>
+          <t>2486529</t>
+        </is>
+      </c>
+      <c r="V491" t="n">
+        <v>63</v>
+      </c>
+      <c r="W491" t="n">
+        <v>74.16</v>
+      </c>
+      <c r="X491" t="n">
+        <v>0.9843581445523194</v>
+      </c>
+      <c r="Y491" t="n">
+        <v>66.16</v>
+      </c>
+      <c r="Z491" t="n">
+        <v>110.3385731559855</v>
+      </c>
+      <c r="AA491" t="n">
+        <v>0.7859281437125749</v>
+      </c>
+      <c r="AB491" t="n">
+        <v>89.79475484606614</v>
+      </c>
+      <c r="AC491" t="n">
+        <v>0.2962962962962963</v>
+      </c>
+      <c r="AD491" t="n">
+        <v>0.7297297297297297</v>
+      </c>
+      <c r="AE491" t="n">
+        <v>0.546875</v>
+      </c>
+      <c r="AF491" t="n">
+        <v>20.54381830991936</v>
+      </c>
+      <c r="AG491" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="AH491" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="AI491" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B492" t="n">
+        <v>31</v>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>200</v>
+      </c>
+      <c r="F492" t="n">
+        <v>81</v>
+      </c>
+      <c r="G492" t="n">
+        <v>12</v>
+      </c>
+      <c r="H492" t="n">
+        <v>31</v>
+      </c>
+      <c r="I492" t="n">
+        <v>12</v>
+      </c>
+      <c r="J492" t="n">
+        <v>31</v>
+      </c>
+      <c r="K492" t="n">
+        <v>21</v>
+      </c>
+      <c r="L492" t="n">
+        <v>28</v>
+      </c>
+      <c r="M492" t="n">
+        <v>11</v>
+      </c>
+      <c r="N492" t="n">
+        <v>26</v>
+      </c>
+      <c r="O492" t="n">
+        <v>21</v>
+      </c>
+      <c r="P492" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q492" t="n">
+        <v>8</v>
+      </c>
+      <c r="R492" t="n">
+        <v>22</v>
+      </c>
+      <c r="S492" t="n">
+        <v>27</v>
+      </c>
+      <c r="T492" t="n">
+        <v>3</v>
+      </c>
+      <c r="U492" t="inlineStr">
+        <is>
+          <t>2486531</t>
+        </is>
+      </c>
+      <c r="V492" t="n">
+        <v>72</v>
+      </c>
+      <c r="W492" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="X492" t="n">
+        <v>0.9839650145772596</v>
+      </c>
+      <c r="Y492" t="n">
+        <v>71.31999999999999</v>
+      </c>
+      <c r="Z492" t="n">
+        <v>113.5726303982053</v>
+      </c>
+      <c r="AA492" t="n">
+        <v>0.9174311926605504</v>
+      </c>
+      <c r="AB492" t="n">
+        <v>102.1566401816118</v>
+      </c>
+      <c r="AC492" t="n">
+        <v>0.3548387096774194</v>
+      </c>
+      <c r="AD492" t="n">
+        <v>0.7647058823529411</v>
+      </c>
+      <c r="AE492" t="n">
+        <v>0.5692307692307692</v>
+      </c>
+      <c r="AF492" t="n">
+        <v>11.41599021659347</v>
+      </c>
+      <c r="AG492" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="AH492" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="AI492" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B493" t="n">
+        <v>31</v>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>200</v>
+      </c>
+      <c r="F493" t="n">
+        <v>73</v>
+      </c>
+      <c r="G493" t="n">
+        <v>14</v>
+      </c>
+      <c r="H493" t="n">
+        <v>26</v>
+      </c>
+      <c r="I493" t="n">
+        <v>10</v>
+      </c>
+      <c r="J493" t="n">
+        <v>34</v>
+      </c>
+      <c r="K493" t="n">
+        <v>15</v>
+      </c>
+      <c r="L493" t="n">
+        <v>20</v>
+      </c>
+      <c r="M493" t="n">
+        <v>11</v>
+      </c>
+      <c r="N493" t="n">
+        <v>26</v>
+      </c>
+      <c r="O493" t="n">
+        <v>10</v>
+      </c>
+      <c r="P493" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q493" t="n">
+        <v>15</v>
+      </c>
+      <c r="R493" t="n">
+        <v>17</v>
+      </c>
+      <c r="S493" t="n">
+        <v>21</v>
+      </c>
+      <c r="T493" t="n">
+        <v>0</v>
+      </c>
+      <c r="U493" t="inlineStr">
+        <is>
+          <t>2486532</t>
+        </is>
+      </c>
+      <c r="V493" t="n">
+        <v>86</v>
+      </c>
+      <c r="W493" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="X493" t="n">
+        <v>0.8711217183770883</v>
+      </c>
+      <c r="Y493" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="Z493" t="n">
+        <v>100.2747252747253</v>
+      </c>
+      <c r="AA493" t="n">
+        <v>1.072854291417166</v>
+      </c>
+      <c r="AB493" t="n">
+        <v>117.550574084199</v>
+      </c>
+      <c r="AC493" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="AD493" t="n">
+        <v>0.7878787878787878</v>
+      </c>
+      <c r="AE493" t="n">
+        <v>0.5362318840579711</v>
+      </c>
+      <c r="AF493" t="n">
+        <v>-17.27584880947374</v>
+      </c>
+      <c r="AG493" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="AH493" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="AI493" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B494" t="n">
+        <v>31</v>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>225</v>
+      </c>
+      <c r="F494" t="n">
+        <v>96</v>
+      </c>
+      <c r="G494" t="n">
+        <v>19</v>
+      </c>
+      <c r="H494" t="n">
+        <v>35</v>
+      </c>
+      <c r="I494" t="n">
+        <v>13</v>
+      </c>
+      <c r="J494" t="n">
+        <v>37</v>
+      </c>
+      <c r="K494" t="n">
+        <v>19</v>
+      </c>
+      <c r="L494" t="n">
+        <v>25</v>
+      </c>
+      <c r="M494" t="n">
+        <v>11</v>
+      </c>
+      <c r="N494" t="n">
+        <v>29</v>
+      </c>
+      <c r="O494" t="n">
+        <v>13</v>
+      </c>
+      <c r="P494" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q494" t="n">
+        <v>16</v>
+      </c>
+      <c r="R494" t="n">
+        <v>19</v>
+      </c>
+      <c r="S494" t="n">
+        <v>21</v>
+      </c>
+      <c r="T494" t="n">
+        <v>2</v>
+      </c>
+      <c r="U494" t="inlineStr">
+        <is>
+          <t>2486530</t>
+        </is>
+      </c>
+      <c r="V494" t="n">
+        <v>99</v>
+      </c>
+      <c r="W494" t="n">
+        <v>99</v>
+      </c>
+      <c r="X494" t="n">
+        <v>0.9696969696969697</v>
+      </c>
+      <c r="Y494" t="n">
+        <v>88</v>
+      </c>
+      <c r="Z494" t="n">
+        <v>109.0909090909091</v>
+      </c>
+      <c r="AA494" t="n">
+        <v>1.07843137254902</v>
+      </c>
+      <c r="AB494" t="n">
+        <v>111.4864864864865</v>
+      </c>
+      <c r="AC494" t="n">
+        <v>0.3142857142857143</v>
+      </c>
+      <c r="AD494" t="n">
+        <v>0.90625</v>
+      </c>
+      <c r="AE494" t="n">
+        <v>0.5970149253731343</v>
+      </c>
+      <c r="AF494" t="n">
+        <v>-2.395577395577391</v>
+      </c>
+      <c r="AG494" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="AH494" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="AI494" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B495" t="n">
+        <v>31</v>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>200</v>
+      </c>
+      <c r="F495" t="n">
+        <v>86</v>
+      </c>
+      <c r="G495" t="n">
+        <v>18</v>
+      </c>
+      <c r="H495" t="n">
+        <v>33</v>
+      </c>
+      <c r="I495" t="n">
+        <v>13</v>
+      </c>
+      <c r="J495" t="n">
+        <v>33</v>
+      </c>
+      <c r="K495" t="n">
+        <v>11</v>
+      </c>
+      <c r="L495" t="n">
+        <v>14</v>
+      </c>
+      <c r="M495" t="n">
+        <v>7</v>
+      </c>
+      <c r="N495" t="n">
+        <v>25</v>
+      </c>
+      <c r="O495" t="n">
+        <v>20</v>
+      </c>
+      <c r="P495" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q495" t="n">
+        <v>8</v>
+      </c>
+      <c r="R495" t="n">
+        <v>21</v>
+      </c>
+      <c r="S495" t="n">
+        <v>17</v>
+      </c>
+      <c r="T495" t="n">
+        <v>2</v>
+      </c>
+      <c r="U495" t="inlineStr">
+        <is>
+          <t>2486532</t>
+        </is>
+      </c>
+      <c r="V495" t="n">
+        <v>73</v>
+      </c>
+      <c r="W495" t="n">
+        <v>80.16</v>
+      </c>
+      <c r="X495" t="n">
+        <v>1.072854291417166</v>
+      </c>
+      <c r="Y495" t="n">
+        <v>73.16</v>
+      </c>
+      <c r="Z495" t="n">
+        <v>117.550574084199</v>
+      </c>
+      <c r="AA495" t="n">
+        <v>0.8711217183770883</v>
+      </c>
+      <c r="AB495" t="n">
+        <v>100.2747252747253</v>
+      </c>
+      <c r="AC495" t="n">
+        <v>0.2121212121212121</v>
+      </c>
+      <c r="AD495" t="n">
+        <v>0.6944444444444444</v>
+      </c>
+      <c r="AE495" t="n">
+        <v>0.463768115942029</v>
+      </c>
+      <c r="AF495" t="n">
+        <v>17.27584880947374</v>
+      </c>
+      <c r="AG495" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="AH495" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="AI495" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B496" t="n">
+        <v>31</v>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>200</v>
+      </c>
+      <c r="F496" t="n">
+        <v>74</v>
+      </c>
+      <c r="G496" t="n">
+        <v>24</v>
+      </c>
+      <c r="H496" t="n">
+        <v>43</v>
+      </c>
+      <c r="I496" t="n">
+        <v>5</v>
+      </c>
+      <c r="J496" t="n">
+        <v>18</v>
+      </c>
+      <c r="K496" t="n">
+        <v>11</v>
+      </c>
+      <c r="L496" t="n">
+        <v>16</v>
+      </c>
+      <c r="M496" t="n">
+        <v>6</v>
+      </c>
+      <c r="N496" t="n">
+        <v>21</v>
+      </c>
+      <c r="O496" t="n">
+        <v>16</v>
+      </c>
+      <c r="P496" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q496" t="n">
+        <v>12</v>
+      </c>
+      <c r="R496" t="n">
+        <v>19</v>
+      </c>
+      <c r="S496" t="n">
+        <v>18</v>
+      </c>
+      <c r="T496" t="n">
+        <v>4</v>
+      </c>
+      <c r="U496" t="inlineStr">
+        <is>
+          <t>2486535</t>
+        </is>
+      </c>
+      <c r="V496" t="n">
+        <v>89</v>
+      </c>
+      <c r="W496" t="n">
+        <v>80.03999999999999</v>
+      </c>
+      <c r="X496" t="n">
+        <v>0.9245377311344328</v>
+      </c>
+      <c r="Y496" t="n">
+        <v>74.03999999999999</v>
+      </c>
+      <c r="Z496" t="n">
+        <v>99.94597514856835</v>
+      </c>
+      <c r="AA496" t="n">
+        <v>1.045091592296853</v>
+      </c>
+      <c r="AB496" t="n">
+        <v>126.8529076396807</v>
+      </c>
+      <c r="AC496" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AD496" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="AE496" t="n">
+        <v>0.4090909090909091</v>
+      </c>
+      <c r="AF496" t="n">
+        <v>-26.90693249111239</v>
+      </c>
+      <c r="AG496" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="AH496" t="inlineStr">
+        <is>
+          <t>ALIMERKA OVIEDO BALONCESTO</t>
+        </is>
+      </c>
+      <c r="AI496" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B497" t="n">
+        <v>31</v>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>200</v>
+      </c>
+      <c r="F497" t="n">
+        <v>93</v>
+      </c>
+      <c r="G497" t="n">
+        <v>13</v>
+      </c>
+      <c r="H497" t="n">
+        <v>35</v>
+      </c>
+      <c r="I497" t="n">
+        <v>13</v>
+      </c>
+      <c r="J497" t="n">
+        <v>25</v>
+      </c>
+      <c r="K497" t="n">
+        <v>28</v>
+      </c>
+      <c r="L497" t="n">
+        <v>31</v>
+      </c>
+      <c r="M497" t="n">
+        <v>7</v>
+      </c>
+      <c r="N497" t="n">
+        <v>18</v>
+      </c>
+      <c r="O497" t="n">
+        <v>21</v>
+      </c>
+      <c r="P497" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q497" t="n">
+        <v>12</v>
+      </c>
+      <c r="R497" t="n">
+        <v>25</v>
+      </c>
+      <c r="S497" t="n">
+        <v>24</v>
+      </c>
+      <c r="T497" t="n">
+        <v>3</v>
+      </c>
+      <c r="U497" t="inlineStr">
+        <is>
+          <t>2486534</t>
+        </is>
+      </c>
+      <c r="V497" t="n">
+        <v>90</v>
+      </c>
+      <c r="W497" t="n">
+        <v>85.64</v>
+      </c>
+      <c r="X497" t="n">
+        <v>1.085941148995796</v>
+      </c>
+      <c r="Y497" t="n">
+        <v>78.64</v>
+      </c>
+      <c r="Z497" t="n">
+        <v>118.2604272634791</v>
+      </c>
+      <c r="AA497" t="n">
+        <v>1.041184636742249</v>
+      </c>
+      <c r="AB497" t="n">
+        <v>122.5490196078431</v>
+      </c>
+      <c r="AC497" t="n">
+        <v>0.2258064516129032</v>
+      </c>
+      <c r="AD497" t="n">
+        <v>0.5806451612903226</v>
+      </c>
+      <c r="AE497" t="n">
+        <v>0.4032258064516129</v>
+      </c>
+      <c r="AF497" t="n">
+        <v>-4.288592344363991</v>
+      </c>
+      <c r="AG497" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="AH497" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="AI497" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B498" t="n">
+        <v>32</v>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>200</v>
+      </c>
+      <c r="F498" t="n">
+        <v>86</v>
+      </c>
+      <c r="G498" t="n">
+        <v>21</v>
+      </c>
+      <c r="H498" t="n">
+        <v>40</v>
+      </c>
+      <c r="I498" t="n">
+        <v>9</v>
+      </c>
+      <c r="J498" t="n">
+        <v>28</v>
+      </c>
+      <c r="K498" t="n">
+        <v>17</v>
+      </c>
+      <c r="L498" t="n">
+        <v>26</v>
+      </c>
+      <c r="M498" t="n">
+        <v>11</v>
+      </c>
+      <c r="N498" t="n">
+        <v>18</v>
+      </c>
+      <c r="O498" t="n">
+        <v>18</v>
+      </c>
+      <c r="P498" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q498" t="n">
+        <v>4</v>
+      </c>
+      <c r="R498" t="n">
+        <v>19</v>
+      </c>
+      <c r="S498" t="n">
+        <v>26</v>
+      </c>
+      <c r="T498" t="n">
+        <v>2</v>
+      </c>
+      <c r="U498" t="inlineStr">
+        <is>
+          <t>2486543</t>
+        </is>
+      </c>
+      <c r="V498" t="n">
+        <v>89</v>
+      </c>
+      <c r="W498" t="n">
+        <v>83.44</v>
+      </c>
+      <c r="X498" t="n">
+        <v>1.030680728667306</v>
+      </c>
+      <c r="Y498" t="n">
+        <v>72.44</v>
+      </c>
+      <c r="Z498" t="n">
+        <v>118.7189398122584</v>
+      </c>
+      <c r="AA498" t="n">
+        <v>1.155244029075805</v>
+      </c>
+      <c r="AB498" t="n">
+        <v>123.5424764019989</v>
+      </c>
+      <c r="AC498" t="n">
+        <v>0.3235294117647059</v>
+      </c>
+      <c r="AD498" t="n">
+        <v>0.7826086956521739</v>
+      </c>
+      <c r="AE498" t="n">
+        <v>0.5087719298245614</v>
+      </c>
+      <c r="AF498" t="n">
+        <v>-4.823536589740471</v>
+      </c>
+      <c r="AG498" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="AH498" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="AI498" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B499" t="n">
+        <v>32</v>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>200</v>
+      </c>
+      <c r="F499" t="n">
+        <v>70</v>
+      </c>
+      <c r="G499" t="n">
+        <v>18</v>
+      </c>
+      <c r="H499" t="n">
+        <v>34</v>
+      </c>
+      <c r="I499" t="n">
+        <v>5</v>
+      </c>
+      <c r="J499" t="n">
+        <v>23</v>
+      </c>
+      <c r="K499" t="n">
+        <v>19</v>
+      </c>
+      <c r="L499" t="n">
+        <v>30</v>
+      </c>
+      <c r="M499" t="n">
+        <v>10</v>
+      </c>
+      <c r="N499" t="n">
+        <v>23</v>
+      </c>
+      <c r="O499" t="n">
+        <v>11</v>
+      </c>
+      <c r="P499" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q499" t="n">
+        <v>9</v>
+      </c>
+      <c r="R499" t="n">
+        <v>27</v>
+      </c>
+      <c r="S499" t="n">
+        <v>28</v>
+      </c>
+      <c r="T499" t="n">
+        <v>2</v>
+      </c>
+      <c r="U499" t="inlineStr">
+        <is>
+          <t>2486537</t>
+        </is>
+      </c>
+      <c r="V499" t="n">
+        <v>73</v>
+      </c>
+      <c r="W499" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="X499" t="n">
+        <v>0.8838383838383838</v>
+      </c>
+      <c r="Y499" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="Z499" t="n">
+        <v>101.1560693641619</v>
+      </c>
+      <c r="AA499" t="n">
+        <v>0.9554973821989529</v>
+      </c>
+      <c r="AB499" t="n">
+        <v>106.7251461988304</v>
+      </c>
+      <c r="AC499" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="AD499" t="n">
+        <v>0.7419354838709677</v>
+      </c>
+      <c r="AE499" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AF499" t="n">
+        <v>-5.56907683466855</v>
+      </c>
+      <c r="AG499" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="AH499" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="AI499" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B500" t="n">
+        <v>32</v>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>200</v>
+      </c>
+      <c r="F500" t="n">
+        <v>70</v>
+      </c>
+      <c r="G500" t="n">
+        <v>13</v>
+      </c>
+      <c r="H500" t="n">
+        <v>34</v>
+      </c>
+      <c r="I500" t="n">
+        <v>11</v>
+      </c>
+      <c r="J500" t="n">
+        <v>30</v>
+      </c>
+      <c r="K500" t="n">
+        <v>11</v>
+      </c>
+      <c r="L500" t="n">
+        <v>21</v>
+      </c>
+      <c r="M500" t="n">
+        <v>11</v>
+      </c>
+      <c r="N500" t="n">
+        <v>25</v>
+      </c>
+      <c r="O500" t="n">
+        <v>15</v>
+      </c>
+      <c r="P500" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q500" t="n">
+        <v>10</v>
+      </c>
+      <c r="R500" t="n">
+        <v>16</v>
+      </c>
+      <c r="S500" t="n">
+        <v>20</v>
+      </c>
+      <c r="T500" t="n">
+        <v>1</v>
+      </c>
+      <c r="U500" t="inlineStr">
+        <is>
+          <t>2486542</t>
+        </is>
+      </c>
+      <c r="V500" t="n">
+        <v>92</v>
+      </c>
+      <c r="W500" t="n">
+        <v>83.24000000000001</v>
+      </c>
+      <c r="X500" t="n">
+        <v>0.8409418548774626</v>
+      </c>
+      <c r="Y500" t="n">
+        <v>72.24000000000001</v>
+      </c>
+      <c r="Z500" t="n">
+        <v>96.89922480620154</v>
+      </c>
+      <c r="AA500" t="n">
+        <v>1.108968177434908</v>
+      </c>
+      <c r="AB500" t="n">
+        <v>127.8488048916064</v>
+      </c>
+      <c r="AC500" t="n">
+        <v>0.2682926829268293</v>
+      </c>
+      <c r="AD500" t="n">
+        <v>0.6944444444444444</v>
+      </c>
+      <c r="AE500" t="n">
+        <v>0.4675324675324675</v>
+      </c>
+      <c r="AF500" t="n">
+        <v>-30.94958008540489</v>
+      </c>
+      <c r="AG500" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="AH500" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="AI500" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B501" t="n">
+        <v>32</v>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>200</v>
+      </c>
+      <c r="F501" t="n">
+        <v>91</v>
+      </c>
+      <c r="G501" t="n">
+        <v>24</v>
+      </c>
+      <c r="H501" t="n">
+        <v>37</v>
+      </c>
+      <c r="I501" t="n">
+        <v>10</v>
+      </c>
+      <c r="J501" t="n">
+        <v>26</v>
+      </c>
+      <c r="K501" t="n">
+        <v>13</v>
+      </c>
+      <c r="L501" t="n">
+        <v>19</v>
+      </c>
+      <c r="M501" t="n">
+        <v>8</v>
+      </c>
+      <c r="N501" t="n">
+        <v>33</v>
+      </c>
+      <c r="O501" t="n">
+        <v>19</v>
+      </c>
+      <c r="P501" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q501" t="n">
+        <v>17</v>
+      </c>
+      <c r="R501" t="n">
+        <v>15</v>
+      </c>
+      <c r="S501" t="n">
+        <v>19</v>
+      </c>
+      <c r="T501" t="n">
+        <v>1</v>
+      </c>
+      <c r="U501" t="inlineStr">
+        <is>
+          <t>2486541</t>
+        </is>
+      </c>
+      <c r="V501" t="n">
+        <v>82</v>
+      </c>
+      <c r="W501" t="n">
+        <v>88.36</v>
+      </c>
+      <c r="X501" t="n">
+        <v>1.02987777274785</v>
+      </c>
+      <c r="Y501" t="n">
+        <v>80.36</v>
+      </c>
+      <c r="Z501" t="n">
+        <v>113.2404181184669</v>
+      </c>
+      <c r="AA501" t="n">
+        <v>0.9860509860509861</v>
+      </c>
+      <c r="AB501" t="n">
+        <v>104.9129989764586</v>
+      </c>
+      <c r="AC501" t="n">
+        <v>0.2962962962962963</v>
+      </c>
+      <c r="AD501" t="n">
+        <v>0.868421052631579</v>
+      </c>
+      <c r="AE501" t="n">
+        <v>0.6307692307692307</v>
+      </c>
+      <c r="AF501" t="n">
+        <v>8.327419142008353</v>
+      </c>
+      <c r="AG501" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="AH501" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="AI501" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B502" t="n">
+        <v>32</v>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>200</v>
+      </c>
+      <c r="F502" t="n">
+        <v>89</v>
+      </c>
+      <c r="G502" t="n">
+        <v>18</v>
+      </c>
+      <c r="H502" t="n">
+        <v>27</v>
+      </c>
+      <c r="I502" t="n">
+        <v>13</v>
+      </c>
+      <c r="J502" t="n">
+        <v>29</v>
+      </c>
+      <c r="K502" t="n">
+        <v>14</v>
+      </c>
+      <c r="L502" t="n">
+        <v>16</v>
+      </c>
+      <c r="M502" t="n">
+        <v>5</v>
+      </c>
+      <c r="N502" t="n">
+        <v>23</v>
+      </c>
+      <c r="O502" t="n">
+        <v>12</v>
+      </c>
+      <c r="P502" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q502" t="n">
+        <v>14</v>
+      </c>
+      <c r="R502" t="n">
+        <v>27</v>
+      </c>
+      <c r="S502" t="n">
+        <v>19</v>
+      </c>
+      <c r="T502" t="n">
+        <v>0</v>
+      </c>
+      <c r="U502" t="inlineStr">
+        <is>
+          <t>2486543</t>
+        </is>
+      </c>
+      <c r="V502" t="n">
+        <v>86</v>
+      </c>
+      <c r="W502" t="n">
+        <v>77.03999999999999</v>
+      </c>
+      <c r="X502" t="n">
+        <v>1.155244029075805</v>
+      </c>
+      <c r="Y502" t="n">
+        <v>72.03999999999999</v>
+      </c>
+      <c r="Z502" t="n">
+        <v>123.5424764019989</v>
+      </c>
+      <c r="AA502" t="n">
+        <v>1.030680728667306</v>
+      </c>
+      <c r="AB502" t="n">
+        <v>118.7189398122584</v>
+      </c>
+      <c r="AC502" t="n">
+        <v>0.2173913043478261</v>
+      </c>
+      <c r="AD502" t="n">
+        <v>0.6764705882352942</v>
+      </c>
+      <c r="AE502" t="n">
+        <v>0.4912280701754386</v>
+      </c>
+      <c r="AF502" t="n">
+        <v>4.823536589740471</v>
+      </c>
+      <c r="AG502" t="inlineStr">
+        <is>
+          <t>GRUPO ALEGA CANTABRIA</t>
+        </is>
+      </c>
+      <c r="AH502" t="inlineStr">
+        <is>
+          <t>CAJA RURAL CB ZAMORA</t>
+        </is>
+      </c>
+      <c r="AI502" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B503" t="n">
+        <v>32</v>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>200</v>
+      </c>
+      <c r="F503" t="n">
+        <v>82</v>
+      </c>
+      <c r="G503" t="n">
+        <v>18</v>
+      </c>
+      <c r="H503" t="n">
+        <v>40</v>
+      </c>
+      <c r="I503" t="n">
+        <v>12</v>
+      </c>
+      <c r="J503" t="n">
+        <v>29</v>
+      </c>
+      <c r="K503" t="n">
+        <v>10</v>
+      </c>
+      <c r="L503" t="n">
+        <v>14</v>
+      </c>
+      <c r="M503" t="n">
+        <v>5</v>
+      </c>
+      <c r="N503" t="n">
+        <v>19</v>
+      </c>
+      <c r="O503" t="n">
+        <v>18</v>
+      </c>
+      <c r="P503" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q503" t="n">
+        <v>8</v>
+      </c>
+      <c r="R503" t="n">
+        <v>19</v>
+      </c>
+      <c r="S503" t="n">
+        <v>15</v>
+      </c>
+      <c r="T503" t="n">
+        <v>4</v>
+      </c>
+      <c r="U503" t="inlineStr">
+        <is>
+          <t>2486541</t>
+        </is>
+      </c>
+      <c r="V503" t="n">
+        <v>91</v>
+      </c>
+      <c r="W503" t="n">
+        <v>83.16</v>
+      </c>
+      <c r="X503" t="n">
+        <v>0.9860509860509861</v>
+      </c>
+      <c r="Y503" t="n">
+        <v>78.16</v>
+      </c>
+      <c r="Z503" t="n">
+        <v>104.9129989764586</v>
+      </c>
+      <c r="AA503" t="n">
+        <v>1.02987777274785</v>
+      </c>
+      <c r="AB503" t="n">
+        <v>113.2404181184669</v>
+      </c>
+      <c r="AC503" t="n">
+        <v>0.131578947368421</v>
+      </c>
+      <c r="AD503" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="AE503" t="n">
+        <v>0.3692307692307693</v>
+      </c>
+      <c r="AF503" t="n">
+        <v>-8.327419142008353</v>
+      </c>
+      <c r="AG503" t="inlineStr">
+        <is>
+          <t>GRUPO CAESA SEGUROS FC CARTAGENA CB</t>
+        </is>
+      </c>
+      <c r="AH503" t="inlineStr">
+        <is>
+          <t>FLEXICAR FUENLABRADA</t>
+        </is>
+      </c>
+      <c r="AI503" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B504" t="n">
+        <v>32</v>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>200</v>
+      </c>
+      <c r="F504" t="n">
+        <v>96</v>
+      </c>
+      <c r="G504" t="n">
+        <v>23</v>
+      </c>
+      <c r="H504" t="n">
+        <v>33</v>
+      </c>
+      <c r="I504" t="n">
+        <v>10</v>
+      </c>
+      <c r="J504" t="n">
+        <v>23</v>
+      </c>
+      <c r="K504" t="n">
+        <v>20</v>
+      </c>
+      <c r="L504" t="n">
+        <v>32</v>
+      </c>
+      <c r="M504" t="n">
+        <v>6</v>
+      </c>
+      <c r="N504" t="n">
+        <v>25</v>
+      </c>
+      <c r="O504" t="n">
+        <v>21</v>
+      </c>
+      <c r="P504" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q504" t="n">
+        <v>16</v>
+      </c>
+      <c r="R504" t="n">
+        <v>27</v>
+      </c>
+      <c r="S504" t="n">
+        <v>29</v>
+      </c>
+      <c r="T504" t="n">
+        <v>3</v>
+      </c>
+      <c r="U504" t="inlineStr">
+        <is>
+          <t>2486544</t>
+        </is>
+      </c>
+      <c r="V504" t="n">
+        <v>81</v>
+      </c>
+      <c r="W504" t="n">
+        <v>86.08</v>
+      </c>
+      <c r="X504" t="n">
+        <v>1.115241635687732</v>
+      </c>
+      <c r="Y504" t="n">
+        <v>80.08</v>
+      </c>
+      <c r="Z504" t="n">
+        <v>119.8801198801199</v>
+      </c>
+      <c r="AA504" t="n">
+        <v>0.8587786259541985</v>
+      </c>
+      <c r="AB504" t="n">
+        <v>99.60649286768323</v>
+      </c>
+      <c r="AC504" t="n">
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="AD504" t="n">
+        <v>0.6578947368421053</v>
+      </c>
+      <c r="AE504" t="n">
+        <v>0.4769230769230769</v>
+      </c>
+      <c r="AF504" t="n">
+        <v>20.27362701243665</v>
+      </c>
+      <c r="AG504" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="AH504" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="AI504" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B505" t="n">
+        <v>32</v>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>200</v>
+      </c>
+      <c r="F505" t="n">
+        <v>73</v>
+      </c>
+      <c r="G505" t="n">
+        <v>12</v>
+      </c>
+      <c r="H505" t="n">
+        <v>27</v>
+      </c>
+      <c r="I505" t="n">
+        <v>7</v>
+      </c>
+      <c r="J505" t="n">
+        <v>26</v>
+      </c>
+      <c r="K505" t="n">
+        <v>28</v>
+      </c>
+      <c r="L505" t="n">
+        <v>35</v>
+      </c>
+      <c r="M505" t="n">
+        <v>8</v>
+      </c>
+      <c r="N505" t="n">
+        <v>25</v>
+      </c>
+      <c r="O505" t="n">
+        <v>13</v>
+      </c>
+      <c r="P505" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q505" t="n">
+        <v>8</v>
+      </c>
+      <c r="R505" t="n">
+        <v>29</v>
+      </c>
+      <c r="S505" t="n">
+        <v>27</v>
+      </c>
+      <c r="T505" t="n">
+        <v>3</v>
+      </c>
+      <c r="U505" t="inlineStr">
+        <is>
+          <t>2486537</t>
+        </is>
+      </c>
+      <c r="V505" t="n">
+        <v>70</v>
+      </c>
+      <c r="W505" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="X505" t="n">
+        <v>0.9554973821989529</v>
+      </c>
+      <c r="Y505" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="Z505" t="n">
+        <v>106.7251461988304</v>
+      </c>
+      <c r="AA505" t="n">
+        <v>0.8838383838383838</v>
+      </c>
+      <c r="AB505" t="n">
+        <v>101.1560693641619</v>
+      </c>
+      <c r="AC505" t="n">
+        <v>0.2580645161290323</v>
+      </c>
+      <c r="AD505" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="AE505" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AF505" t="n">
+        <v>5.56907683466855</v>
+      </c>
+      <c r="AG505" t="inlineStr">
+        <is>
+          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="AH505" t="inlineStr">
+        <is>
+          <t>HESTIA MENORCA</t>
+        </is>
+      </c>
+      <c r="AI505" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B506" t="n">
+        <v>32</v>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>200</v>
+      </c>
+      <c r="F506" t="n">
+        <v>68</v>
+      </c>
+      <c r="G506" t="n">
+        <v>11</v>
+      </c>
+      <c r="H506" t="n">
+        <v>35</v>
+      </c>
+      <c r="I506" t="n">
+        <v>11</v>
+      </c>
+      <c r="J506" t="n">
+        <v>33</v>
+      </c>
+      <c r="K506" t="n">
+        <v>13</v>
+      </c>
+      <c r="L506" t="n">
+        <v>20</v>
+      </c>
+      <c r="M506" t="n">
+        <v>15</v>
+      </c>
+      <c r="N506" t="n">
+        <v>29</v>
+      </c>
+      <c r="O506" t="n">
+        <v>16</v>
+      </c>
+      <c r="P506" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q506" t="n">
+        <v>11</v>
+      </c>
+      <c r="R506" t="n">
+        <v>22</v>
+      </c>
+      <c r="S506" t="n">
+        <v>21</v>
+      </c>
+      <c r="T506" t="n">
+        <v>2</v>
+      </c>
+      <c r="U506" t="inlineStr">
+        <is>
+          <t>2486538</t>
+        </is>
+      </c>
+      <c r="V506" t="n">
+        <v>77</v>
+      </c>
+      <c r="W506" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="X506" t="n">
+        <v>0.7744874715261959</v>
+      </c>
+      <c r="Y506" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="Z506" t="n">
+        <v>93.40659340659342</v>
+      </c>
+      <c r="AA506" t="n">
+        <v>0.918854415274463</v>
+      </c>
+      <c r="AB506" t="n">
+        <v>104.3360433604336</v>
+      </c>
+      <c r="AC506" t="n">
+        <v>0.3488372093023256</v>
+      </c>
+      <c r="AD506" t="n">
+        <v>0.7435897435897436</v>
+      </c>
+      <c r="AE506" t="n">
+        <v>0.5365853658536586</v>
+      </c>
+      <c r="AF506" t="n">
+        <v>-10.92944995384019</v>
+      </c>
+      <c r="AG506" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="AH506" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="AI506" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B507" t="n">
+        <v>32</v>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>200</v>
+      </c>
+      <c r="F507" t="n">
+        <v>81</v>
+      </c>
+      <c r="G507" t="n">
+        <v>20</v>
+      </c>
+      <c r="H507" t="n">
+        <v>35</v>
+      </c>
+      <c r="I507" t="n">
+        <v>10</v>
+      </c>
+      <c r="J507" t="n">
+        <v>25</v>
+      </c>
+      <c r="K507" t="n">
+        <v>11</v>
+      </c>
+      <c r="L507" t="n">
+        <v>17</v>
+      </c>
+      <c r="M507" t="n">
+        <v>4</v>
+      </c>
+      <c r="N507" t="n">
+        <v>24</v>
+      </c>
+      <c r="O507" t="n">
+        <v>29</v>
+      </c>
+      <c r="P507" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q507" t="n">
+        <v>11</v>
+      </c>
+      <c r="R507" t="n">
+        <v>17</v>
+      </c>
+      <c r="S507" t="n">
+        <v>20</v>
+      </c>
+      <c r="T507" t="n">
+        <v>3</v>
+      </c>
+      <c r="U507" t="inlineStr">
+        <is>
+          <t>2486539</t>
+        </is>
+      </c>
+      <c r="V507" t="n">
+        <v>92</v>
+      </c>
+      <c r="W507" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="X507" t="n">
+        <v>1.032110091743119</v>
+      </c>
+      <c r="Y507" t="n">
+        <v>74.48</v>
+      </c>
+      <c r="Z507" t="n">
+        <v>108.7540279269602</v>
+      </c>
+      <c r="AA507" t="n">
+        <v>0.9603340292275574</v>
+      </c>
+      <c r="AB507" t="n">
+        <v>113.8613861386139</v>
+      </c>
+      <c r="AC507" t="n">
+        <v>0.1379310344827586</v>
+      </c>
+      <c r="AD507" t="n">
+        <v>0.6153846153846154</v>
+      </c>
+      <c r="AE507" t="n">
+        <v>0.4117647058823529</v>
+      </c>
+      <c r="AF507" t="n">
+        <v>-5.107358211653619</v>
+      </c>
+      <c r="AG507" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="AH507" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="AI507" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B508" t="n">
+        <v>32</v>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>200</v>
+      </c>
+      <c r="F508" t="n">
+        <v>92</v>
+      </c>
+      <c r="G508" t="n">
+        <v>24</v>
+      </c>
+      <c r="H508" t="n">
+        <v>51</v>
+      </c>
+      <c r="I508" t="n">
+        <v>10</v>
+      </c>
+      <c r="J508" t="n">
+        <v>27</v>
+      </c>
+      <c r="K508" t="n">
+        <v>14</v>
+      </c>
+      <c r="L508" t="n">
+        <v>20</v>
+      </c>
+      <c r="M508" t="n">
+        <v>15</v>
+      </c>
+      <c r="N508" t="n">
+        <v>25</v>
+      </c>
+      <c r="O508" t="n">
+        <v>22</v>
+      </c>
+      <c r="P508" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q508" t="n">
+        <v>9</v>
+      </c>
+      <c r="R508" t="n">
+        <v>20</v>
+      </c>
+      <c r="S508" t="n">
+        <v>17</v>
+      </c>
+      <c r="T508" t="n">
+        <v>1</v>
+      </c>
+      <c r="U508" t="inlineStr">
+        <is>
+          <t>2486539</t>
+        </is>
+      </c>
+      <c r="V508" t="n">
+        <v>81</v>
+      </c>
+      <c r="W508" t="n">
+        <v>95.8</v>
+      </c>
+      <c r="X508" t="n">
+        <v>0.9603340292275574</v>
+      </c>
+      <c r="Y508" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="Z508" t="n">
+        <v>113.8613861386139</v>
+      </c>
+      <c r="AA508" t="n">
+        <v>1.032110091743119</v>
+      </c>
+      <c r="AB508" t="n">
+        <v>108.7540279269602</v>
+      </c>
+      <c r="AC508" t="n">
+        <v>0.3846153846153846</v>
+      </c>
+      <c r="AD508" t="n">
+        <v>0.8620689655172413</v>
+      </c>
+      <c r="AE508" t="n">
+        <v>0.5882352941176471</v>
+      </c>
+      <c r="AF508" t="n">
+        <v>5.107358211653619</v>
+      </c>
+      <c r="AG508" t="inlineStr">
+        <is>
+          <t>INVEREADY GIPUZKOA</t>
+        </is>
+      </c>
+      <c r="AH508" t="inlineStr">
+        <is>
+          <t>LEYMA CORUÑA</t>
+        </is>
+      </c>
+      <c r="AI508" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B509" t="n">
+        <v>32</v>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>200</v>
+      </c>
+      <c r="F509" t="n">
+        <v>81</v>
+      </c>
+      <c r="G509" t="n">
+        <v>13</v>
+      </c>
+      <c r="H509" t="n">
+        <v>30</v>
+      </c>
+      <c r="I509" t="n">
+        <v>11</v>
+      </c>
+      <c r="J509" t="n">
+        <v>37</v>
+      </c>
+      <c r="K509" t="n">
+        <v>22</v>
+      </c>
+      <c r="L509" t="n">
+        <v>28</v>
+      </c>
+      <c r="M509" t="n">
+        <v>13</v>
+      </c>
+      <c r="N509" t="n">
+        <v>21</v>
+      </c>
+      <c r="O509" t="n">
+        <v>12</v>
+      </c>
+      <c r="P509" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q509" t="n">
+        <v>15</v>
+      </c>
+      <c r="R509" t="n">
+        <v>29</v>
+      </c>
+      <c r="S509" t="n">
+        <v>26</v>
+      </c>
+      <c r="T509" t="n">
+        <v>0</v>
+      </c>
+      <c r="U509" t="inlineStr">
+        <is>
+          <t>2486544</t>
+        </is>
+      </c>
+      <c r="V509" t="n">
+        <v>96</v>
+      </c>
+      <c r="W509" t="n">
+        <v>94.31999999999999</v>
+      </c>
+      <c r="X509" t="n">
+        <v>0.8587786259541985</v>
+      </c>
+      <c r="Y509" t="n">
+        <v>81.31999999999999</v>
+      </c>
+      <c r="Z509" t="n">
+        <v>99.60649286768323</v>
+      </c>
+      <c r="AA509" t="n">
+        <v>1.115241635687732</v>
+      </c>
+      <c r="AB509" t="n">
+        <v>119.8801198801199</v>
+      </c>
+      <c r="AC509" t="n">
+        <v>0.3421052631578947</v>
+      </c>
+      <c r="AD509" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="AE509" t="n">
+        <v>0.5230769230769231</v>
+      </c>
+      <c r="AF509" t="n">
+        <v>-20.27362701243665</v>
+      </c>
+      <c r="AG509" t="inlineStr">
+        <is>
+          <t>GRUPO URETA TIZONA BURGOS</t>
+        </is>
+      </c>
+      <c r="AH509" t="inlineStr">
+        <is>
+          <t>MELILLA CIUDAD DEL DEPORTE</t>
+        </is>
+      </c>
+      <c r="AI509" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B510" t="n">
+        <v>32</v>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>200</v>
+      </c>
+      <c r="F510" t="n">
+        <v>89</v>
+      </c>
+      <c r="G510" t="n">
+        <v>17</v>
+      </c>
+      <c r="H510" t="n">
+        <v>30</v>
+      </c>
+      <c r="I510" t="n">
+        <v>13</v>
+      </c>
+      <c r="J510" t="n">
+        <v>35</v>
+      </c>
+      <c r="K510" t="n">
+        <v>16</v>
+      </c>
+      <c r="L510" t="n">
+        <v>20</v>
+      </c>
+      <c r="M510" t="n">
+        <v>14</v>
+      </c>
+      <c r="N510" t="n">
+        <v>20</v>
+      </c>
+      <c r="O510" t="n">
+        <v>14</v>
+      </c>
+      <c r="P510" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q510" t="n">
+        <v>9</v>
+      </c>
+      <c r="R510" t="n">
+        <v>23</v>
+      </c>
+      <c r="S510" t="n">
+        <v>22</v>
+      </c>
+      <c r="T510" t="n">
+        <v>2</v>
+      </c>
+      <c r="U510" t="inlineStr">
+        <is>
+          <t>2486540</t>
+        </is>
+      </c>
+      <c r="V510" t="n">
+        <v>79</v>
+      </c>
+      <c r="W510" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="X510" t="n">
+        <v>1.07487922705314</v>
+      </c>
+      <c r="Y510" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="Z510" t="n">
+        <v>129.3604651162791</v>
+      </c>
+      <c r="AA510" t="n">
+        <v>1.004067107269954</v>
+      </c>
+      <c r="AB510" t="n">
+        <v>108.695652173913</v>
+      </c>
+      <c r="AC510" t="n">
+        <v>0.4242424242424243</v>
+      </c>
+      <c r="AD510" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="AE510" t="n">
+        <v>0.576271186440678</v>
+      </c>
+      <c r="AF510" t="n">
+        <v>20.66481294236604</v>
+      </c>
+      <c r="AG510" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="AH510" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="AI510" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B511" t="n">
+        <v>32</v>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>200</v>
+      </c>
+      <c r="F511" t="n">
+        <v>79</v>
+      </c>
+      <c r="G511" t="n">
+        <v>15</v>
+      </c>
+      <c r="H511" t="n">
+        <v>23</v>
+      </c>
+      <c r="I511" t="n">
+        <v>11</v>
+      </c>
+      <c r="J511" t="n">
+        <v>30</v>
+      </c>
+      <c r="K511" t="n">
+        <v>16</v>
+      </c>
+      <c r="L511" t="n">
+        <v>22</v>
+      </c>
+      <c r="M511" t="n">
+        <v>6</v>
+      </c>
+      <c r="N511" t="n">
+        <v>19</v>
+      </c>
+      <c r="O511" t="n">
+        <v>23</v>
+      </c>
+      <c r="P511" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q511" t="n">
+        <v>16</v>
+      </c>
+      <c r="R511" t="n">
+        <v>22</v>
+      </c>
+      <c r="S511" t="n">
+        <v>22</v>
+      </c>
+      <c r="T511" t="n">
+        <v>0</v>
+      </c>
+      <c r="U511" t="inlineStr">
+        <is>
+          <t>2486540</t>
+        </is>
+      </c>
+      <c r="V511" t="n">
+        <v>89</v>
+      </c>
+      <c r="W511" t="n">
+        <v>78.68000000000001</v>
+      </c>
+      <c r="X511" t="n">
+        <v>1.004067107269954</v>
+      </c>
+      <c r="Y511" t="n">
+        <v>72.68000000000001</v>
+      </c>
+      <c r="Z511" t="n">
+        <v>108.695652173913</v>
+      </c>
+      <c r="AA511" t="n">
+        <v>1.07487922705314</v>
+      </c>
+      <c r="AB511" t="n">
+        <v>129.3604651162791</v>
+      </c>
+      <c r="AC511" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="AD511" t="n">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="AE511" t="n">
+        <v>0.423728813559322</v>
+      </c>
+      <c r="AF511" t="n">
+        <v>-20.66481294236604</v>
+      </c>
+      <c r="AG511" t="inlineStr">
+        <is>
+          <t>MOVISTAR ESTUDIANTES</t>
+        </is>
+      </c>
+      <c r="AH511" t="inlineStr">
+        <is>
+          <t>MONBUS OBRADOIRO</t>
+        </is>
+      </c>
+      <c r="AI511" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B512" t="n">
+        <v>32</v>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>200</v>
+      </c>
+      <c r="F512" t="n">
+        <v>77</v>
+      </c>
+      <c r="G512" t="n">
+        <v>16</v>
+      </c>
+      <c r="H512" t="n">
+        <v>34</v>
+      </c>
+      <c r="I512" t="n">
+        <v>9</v>
+      </c>
+      <c r="J512" t="n">
+        <v>32</v>
+      </c>
+      <c r="K512" t="n">
+        <v>18</v>
+      </c>
+      <c r="L512" t="n">
+        <v>20</v>
+      </c>
+      <c r="M512" t="n">
+        <v>10</v>
+      </c>
+      <c r="N512" t="n">
+        <v>28</v>
+      </c>
+      <c r="O512" t="n">
+        <v>12</v>
+      </c>
+      <c r="P512" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q512" t="n">
+        <v>9</v>
+      </c>
+      <c r="R512" t="n">
+        <v>21</v>
+      </c>
+      <c r="S512" t="n">
+        <v>20</v>
+      </c>
+      <c r="T512" t="n">
+        <v>5</v>
+      </c>
+      <c r="U512" t="inlineStr">
+        <is>
+          <t>2486538</t>
+        </is>
+      </c>
+      <c r="V512" t="n">
+        <v>68</v>
+      </c>
+      <c r="W512" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="X512" t="n">
+        <v>0.918854415274463</v>
+      </c>
+      <c r="Y512" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="Z512" t="n">
+        <v>104.3360433604336</v>
+      </c>
+      <c r="AA512" t="n">
+        <v>0.7744874715261959</v>
+      </c>
+      <c r="AB512" t="n">
+        <v>93.40659340659342</v>
+      </c>
+      <c r="AC512" t="n">
+        <v>0.2564102564102564</v>
+      </c>
+      <c r="AD512" t="n">
+        <v>0.6511627906976745</v>
+      </c>
+      <c r="AE512" t="n">
+        <v>0.4634146341463415</v>
+      </c>
+      <c r="AF512" t="n">
+        <v>10.92944995384019</v>
+      </c>
+      <c r="AG512" t="inlineStr">
+        <is>
+          <t>HLA ALICANTE</t>
+        </is>
+      </c>
+      <c r="AH512" t="inlineStr">
+        <is>
+          <t>PALMER BASKET MALLORCA PALMA</t>
+        </is>
+      </c>
+      <c r="AI512" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Liga Regular Único</t>
+        </is>
+      </c>
+      <c r="B513" t="n">
+        <v>32</v>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>200</v>
+      </c>
+      <c r="F513" t="n">
+        <v>92</v>
+      </c>
+      <c r="G513" t="n">
+        <v>26</v>
+      </c>
+      <c r="H513" t="n">
+        <v>43</v>
+      </c>
+      <c r="I513" t="n">
+        <v>12</v>
+      </c>
+      <c r="J513" t="n">
+        <v>29</v>
+      </c>
+      <c r="K513" t="n">
+        <v>4</v>
+      </c>
+      <c r="L513" t="n">
+        <v>9</v>
+      </c>
+      <c r="M513" t="n">
+        <v>11</v>
+      </c>
+      <c r="N513" t="n">
+        <v>30</v>
+      </c>
+      <c r="O513" t="n">
+        <v>24</v>
+      </c>
+      <c r="P513" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q513" t="n">
+        <v>7</v>
+      </c>
+      <c r="R513" t="n">
+        <v>20</v>
+      </c>
+      <c r="S513" t="n">
+        <v>16</v>
+      </c>
+      <c r="T513" t="n">
+        <v>1</v>
+      </c>
+      <c r="U513" t="inlineStr">
+        <is>
+          <t>2486542</t>
+        </is>
+      </c>
+      <c r="V513" t="n">
+        <v>70</v>
+      </c>
+      <c r="W513" t="n">
+        <v>82.96000000000001</v>
+      </c>
+      <c r="X513" t="n">
+        <v>1.108968177434908</v>
+      </c>
+      <c r="Y513" t="n">
+        <v>71.96000000000001</v>
+      </c>
+      <c r="Z513" t="n">
+        <v>127.8488048916064</v>
+      </c>
+      <c r="AA513" t="n">
+        <v>0.8409418548774626</v>
+      </c>
+      <c r="AB513" t="n">
+        <v>96.89922480620154</v>
+      </c>
+      <c r="AC513" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="AD513" t="n">
+        <v>0.7317073170731707</v>
+      </c>
+      <c r="AE513" t="n">
+        <v>0.5324675324675324</v>
+      </c>
+      <c r="AF513" t="n">
+        <v>30.94958008540489</v>
+      </c>
+      <c r="AG513" t="inlineStr">
+        <is>
+          <t>FIBWI MALLORCA BASQUET PALMA</t>
+        </is>
+      </c>
+      <c r="AH513" t="inlineStr">
+        <is>
+          <t>SÚPER AGROPAL PALENCIA</t>
+        </is>
+      </c>
+      <c r="AI513" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>